<commit_message>
report: update 2026-09-09 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46270</v>
+        <v>46274</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发2次，迟发1次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-09-10 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46274</v>
+        <v>46275</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">

</xml_diff>

<commit_message>
report: update 2026-09-13 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46275</v>
+        <v>46278</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发1次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-09-14 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46278</v>
+        <v>46279</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4411,7 +4411,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发3次，迟发2次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-09-17 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46279</v>
+        <v>46282</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3367,7 +3367,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D17" s="68" t="n"/>
+      <c r="D17" s="68" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E17" s="69" t="n"/>
       <c r="F17" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-09-18 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46282</v>
+        <v>46283</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3888,7 +3888,7 @@
       </c>
       <c r="D36" s="73" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发1次</t>
+          <t>累计未发4次，迟发1次</t>
         </is>
       </c>
       <c r="E36" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-09-20 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O65"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46283</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46285</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2812,7 +2812,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3073,17 +3073,17 @@
         <f>COUNTIFS($A:$A,$G9,$C:$C,"&lt;&gt;新中心")</f>
         <v/>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="L9" s="0" t="inlineStr">
         <is>
           <t>汇总</t>
         </is>
       </c>
-      <c r="M9">
+      <c r="M9" s="0">
         <f>SUM(M3:M8)</f>
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3175,7 +3175,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3217,7 +3217,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3259,7 +3259,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3296,7 +3296,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3327,7 +3327,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3360,7 +3360,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3414,7 +3414,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3522,7 +3522,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3547,7 +3547,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3572,7 +3572,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3599,7 +3599,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3630,7 +3630,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3684,7 +3684,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3713,7 +3713,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3742,7 +3742,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3771,7 +3771,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3796,7 +3796,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3821,7 +3821,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3850,7 +3850,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3879,7 +3879,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3908,7 +3908,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3933,7 +3933,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -3962,7 +3962,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -3991,7 +3991,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4016,7 +4016,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4045,7 +4045,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4074,7 +4074,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4103,7 +4103,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4128,7 +4128,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4157,7 +4157,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4182,7 +4182,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4211,7 +4211,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4240,7 +4240,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4258,7 +4258,7 @@
       </c>
       <c r="D49" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E49" s="69" t="n"/>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4294,7 +4294,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4323,7 +4323,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4348,7 +4348,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4377,7 +4377,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4406,7 +4406,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4435,7 +4435,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4460,7 +4460,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4489,7 +4489,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4518,7 +4518,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4547,7 +4547,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4576,7 +4576,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4629,7 +4629,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4657,7 +4657,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4684,7 +4684,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="65" s="53">
       <c r="A65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -4706,206 +4706,206 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="53"/>
-    <row r="67" ht="16" customHeight="1" s="53"/>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+    <row customHeight="1" ht="16" r="66" s="53"/>
+    <row customHeight="1" ht="16" r="67" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4918,17 +4918,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -4951,7 +4951,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -5037,7 +5037,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5080,7 +5080,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5125,7 +5125,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5162,7 +5162,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5207,7 +5207,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5246,7 +5246,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5283,7 +5283,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5312,7 +5312,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5351,7 +5351,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5388,7 +5388,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5425,7 +5425,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5464,7 +5464,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5501,7 +5501,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5528,7 +5528,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5556,7 +5556,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5584,7 +5584,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5612,7 +5612,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5642,7 +5642,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5672,7 +5672,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5708,7 +5708,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5736,7 +5736,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5766,7 +5766,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5804,7 +5804,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5834,7 +5834,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5866,7 +5866,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5900,7 +5900,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5932,7 +5932,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5960,7 +5960,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5996,7 +5996,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6023,7 +6023,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6055,7 +6055,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6087,7 +6087,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6112,7 +6112,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6142,7 +6142,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6172,7 +6172,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6206,7 +6206,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6236,7 +6236,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6264,7 +6264,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6292,7 +6292,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6320,7 +6320,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6348,7 +6348,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6376,7 +6376,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6404,7 +6404,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6432,7 +6432,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6460,7 +6460,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6498,7 +6498,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6528,7 +6528,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6564,7 +6564,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6598,7 +6598,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6634,7 +6634,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6666,7 +6666,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7314,7 +7314,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7327,17 +7327,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7360,7 +7360,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7446,7 +7446,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7492,7 +7492,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7529,7 +7529,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7575,7 +7575,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7621,7 +7621,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7669,7 +7669,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7706,7 +7706,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7743,7 +7743,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7791,7 +7791,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7837,7 +7837,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7874,7 +7874,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7911,7 +7911,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7957,7 +7957,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7985,7 +7985,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8013,7 +8013,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8041,7 +8041,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8069,7 +8069,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8097,7 +8097,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8125,7 +8125,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8153,7 +8153,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8181,7 +8181,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8209,7 +8209,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8237,7 +8237,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8265,7 +8265,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8293,7 +8293,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8321,7 +8321,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8351,7 +8351,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8379,7 +8379,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8407,7 +8407,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8435,7 +8435,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8463,7 +8463,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8491,7 +8491,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8519,7 +8519,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8549,7 +8549,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8577,7 +8577,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8605,7 +8605,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8633,7 +8633,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8661,7 +8661,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8691,7 +8691,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8723,7 +8723,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8751,7 +8751,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8779,7 +8779,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8807,7 +8807,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8835,7 +8835,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8863,7 +8863,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8895,7 +8895,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8927,7 +8927,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9603,7 +9603,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9614,16 +9614,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9633,7 +9633,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9678,7 +9678,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9724,7 +9724,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9769,7 +9769,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9818,7 +9818,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9867,7 +9867,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9909,7 +9909,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9944,7 +9944,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9984,7 +9984,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10020,7 +10020,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10056,7 +10056,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10092,7 +10092,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10133,7 +10133,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10164,7 +10164,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10186,7 +10186,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10203,7 +10203,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10220,7 +10220,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10242,7 +10242,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10259,7 +10259,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10277,7 +10277,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10299,7 +10299,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10321,7 +10321,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10343,7 +10343,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10365,7 +10365,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10383,7 +10383,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10405,7 +10405,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10427,7 +10427,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10449,7 +10449,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10471,7 +10471,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10493,7 +10493,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10515,7 +10515,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10542,7 +10542,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10564,7 +10564,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10586,7 +10586,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10608,7 +10608,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10630,7 +10630,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10652,7 +10652,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10674,7 +10674,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10691,7 +10691,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10713,7 +10713,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10731,7 +10731,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10753,7 +10753,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10771,7 +10771,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10789,7 +10789,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10811,7 +10811,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10833,7 +10833,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10855,7 +10855,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10877,7 +10877,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10899,7 +10899,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10922,7 +10922,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10944,7 +10944,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10966,7 +10966,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10988,7 +10988,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -11010,7 +11010,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -11032,7 +11032,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11054,7 +11054,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11072,7 +11072,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11083,18 +11083,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11136,7 +11136,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11179,7 +11179,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11212,7 +11212,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11250,7 +11250,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11293,7 +11293,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11326,7 +11326,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11355,7 +11355,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11385,7 +11385,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11410,7 +11410,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11435,7 +11435,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11465,7 +11465,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11490,7 +11490,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11520,7 +11520,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11540,7 +11540,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11570,7 +11570,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11595,7 +11595,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11630,7 +11630,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11665,7 +11665,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11690,7 +11690,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11720,7 +11720,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11750,7 +11750,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11780,7 +11780,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11810,7 +11810,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11840,7 +11840,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11870,7 +11870,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11895,7 +11895,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11925,7 +11925,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -11955,7 +11955,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -11985,7 +11985,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -12020,7 +12020,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -12050,7 +12050,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12080,7 +12080,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12110,7 +12110,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12140,7 +12140,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12170,7 +12170,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12200,7 +12200,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12235,7 +12235,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12266,6 +12266,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-09-21 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46285</v>
+        <v>46286</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3812,7 +3812,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D33" s="71" t="n"/>
+      <c r="D33" s="71" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E33" s="69" t="n"/>
       <c r="F33" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-09-24 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46286</v>
+        <v>46289</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发2次</t>
+          <t>累计未发3次，迟发3次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-09-25 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46289</v>
+        <v>46290</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="D33" s="71" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>迟发2次</t>
         </is>
       </c>
       <c r="E33" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-09-27 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46290</v>
+        <v>46292</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3147,7 +3147,7 @@
       </c>
       <c r="D11" s="71" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>迟发2次</t>
         </is>
       </c>
       <c r="E11" s="69" t="n"/>
@@ -3378,7 +3378,7 @@
       </c>
       <c r="D17" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E17" s="69" t="n"/>
@@ -3984,7 +3984,7 @@
       </c>
       <c r="D39" s="70" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E39" s="69" t="n"/>
@@ -4096,7 +4096,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发3次</t>
+          <t>累计未发3次，迟发3次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>
@@ -4399,7 +4399,7 @@
       </c>
       <c r="D54" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E54" s="69" t="n"/>
@@ -4540,7 +4540,7 @@
       </c>
       <c r="D59" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发2次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E59" s="69" t="n"/>
@@ -4651,7 +4651,7 @@
       </c>
       <c r="D63" s="68" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E63" s="69" t="n"/>
@@ -4679,7 +4679,7 @@
       </c>
       <c r="D64" s="0" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发1次</t>
+          <t>累计未发1次，迟发2次</t>
         </is>
       </c>
       <c r="F64" s="0" t="inlineStr">

</xml_diff>

<commit_message>
report: update 2026-10-10 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46292</v>
+        <v>46305</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -2766,7 +2766,7 @@
       </c>
       <c r="D4" s="71" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发2次，迟发1次</t>
         </is>
       </c>
       <c r="E4" s="69" t="n"/>
@@ -3233,7 +3233,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D13" s="70" t="n"/>
+      <c r="D13" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E13" s="70" t="n"/>
       <c r="F13" s="63" t="inlineStr">
         <is>
@@ -3343,7 +3347,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D16" s="70" t="n"/>
+      <c r="D16" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E16" s="69" t="n"/>
       <c r="F16" s="63" t="inlineStr">
         <is>
@@ -3843,7 +3851,7 @@
       </c>
       <c r="D34" s="71" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发1次</t>
+          <t>累计未发3次，迟发1次</t>
         </is>
       </c>
       <c r="E34" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-10-13 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O66"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46305</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46308</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2812,7 +2812,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3083,7 +3083,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3175,7 +3175,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3217,7 +3217,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3263,7 +3263,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3300,7 +3300,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3331,7 +3331,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3521,7 +3521,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D22" s="70" t="n"/>
+      <c r="D22" s="70" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E22" s="69" t="n"/>
       <c r="F22" s="63" t="inlineStr">
         <is>
@@ -3530,7 +3534,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3555,7 +3559,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3580,7 +3584,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3607,7 +3611,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3638,7 +3642,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3667,7 +3671,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3692,7 +3696,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3721,7 +3725,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3750,7 +3754,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3779,7 +3783,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3804,7 +3808,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3833,7 +3837,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3862,7 +3866,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3891,7 +3895,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3920,7 +3924,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3945,7 +3949,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -3974,7 +3978,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4003,7 +4007,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4028,7 +4032,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4057,7 +4061,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4086,7 +4090,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4115,7 +4119,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4140,7 +4144,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4169,7 +4173,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4194,7 +4198,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4223,7 +4227,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4241,7 +4245,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发1次</t>
+          <t>累计未发1次，迟发2次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4252,7 +4256,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4281,7 +4285,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4306,7 +4310,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4335,7 +4339,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4360,7 +4364,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4389,7 +4393,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4418,7 +4422,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4447,7 +4451,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4472,7 +4476,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4501,7 +4505,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4530,7 +4534,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4559,7 +4563,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4588,7 +4592,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4617,7 +4621,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4641,7 +4645,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4669,7 +4673,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4696,7 +4700,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="65" s="53">
       <c r="A65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -4718,222 +4722,222 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="53">
-      <c r="A66" t="inlineStr">
+    <row customHeight="1" ht="16" r="66" s="53">
+      <c r="A66" s="0" t="inlineStr">
         <is>
           <t>粤西区</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B66" s="0" t="inlineStr">
         <is>
           <t>广州文冲中心</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>是</t>
-        </is>
-      </c>
-    </row>
-    <row r="67" ht="16" customHeight="1" s="53"/>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+      <c r="C66" s="0" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="16" r="67" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4946,17 +4950,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -4979,7 +4983,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -5065,7 +5069,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5108,7 +5112,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5153,7 +5157,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5190,7 +5194,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5235,7 +5239,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5274,7 +5278,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5311,7 +5315,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5340,7 +5344,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5379,7 +5383,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5416,7 +5420,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5453,7 +5457,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5492,7 +5496,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5529,7 +5533,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5556,7 +5560,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5584,7 +5588,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5612,7 +5616,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5640,7 +5644,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5670,7 +5674,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5700,7 +5704,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5736,7 +5740,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5764,7 +5768,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5794,7 +5798,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5832,7 +5836,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5862,7 +5866,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5894,7 +5898,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5928,7 +5932,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5960,7 +5964,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -5988,7 +5992,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6024,7 +6028,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6051,7 +6055,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6083,7 +6087,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6115,7 +6119,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6140,7 +6144,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6170,7 +6174,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6200,7 +6204,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6234,7 +6238,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6264,7 +6268,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6292,7 +6296,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6320,7 +6324,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6348,7 +6352,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6376,7 +6380,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6404,7 +6408,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6432,7 +6436,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6460,7 +6464,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6488,7 +6492,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6526,7 +6530,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6556,7 +6560,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6592,7 +6596,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6626,7 +6630,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6662,7 +6666,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6694,7 +6698,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7342,7 +7346,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7355,17 +7359,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7388,7 +7392,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7474,7 +7478,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7520,7 +7524,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7557,7 +7561,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7603,7 +7607,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7649,7 +7653,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7697,7 +7701,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7734,7 +7738,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7771,7 +7775,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7819,7 +7823,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7865,7 +7869,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7902,7 +7906,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7939,7 +7943,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7985,7 +7989,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8013,7 +8017,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8041,7 +8045,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8069,7 +8073,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8097,7 +8101,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8125,7 +8129,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8153,7 +8157,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8181,7 +8185,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8209,7 +8213,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8237,7 +8241,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8265,7 +8269,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8293,7 +8297,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8321,7 +8325,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8349,7 +8353,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8379,7 +8383,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8407,7 +8411,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8435,7 +8439,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8463,7 +8467,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8491,7 +8495,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8519,7 +8523,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8547,7 +8551,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8577,7 +8581,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8605,7 +8609,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8633,7 +8637,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8661,7 +8665,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8689,7 +8693,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8719,7 +8723,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8751,7 +8755,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8779,7 +8783,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8807,7 +8811,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8835,7 +8839,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8863,7 +8867,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8891,7 +8895,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8923,7 +8927,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8955,7 +8959,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9631,7 +9635,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9642,16 +9646,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9661,7 +9665,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9706,7 +9710,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9752,7 +9756,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9797,7 +9801,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9846,7 +9850,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9895,7 +9899,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9937,7 +9941,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -9972,7 +9976,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10012,7 +10016,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10048,7 +10052,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10084,7 +10088,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10120,7 +10124,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10161,7 +10165,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10192,7 +10196,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10214,7 +10218,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10231,7 +10235,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10248,7 +10252,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10270,7 +10274,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10287,7 +10291,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10305,7 +10309,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10327,7 +10331,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10349,7 +10353,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10371,7 +10375,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10393,7 +10397,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10411,7 +10415,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10433,7 +10437,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10455,7 +10459,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10477,7 +10481,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10499,7 +10503,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10521,7 +10525,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10543,7 +10547,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10570,7 +10574,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10592,7 +10596,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10614,7 +10618,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10636,7 +10640,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10658,7 +10662,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10680,7 +10684,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10702,7 +10706,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10719,7 +10723,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10741,7 +10745,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10759,7 +10763,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10781,7 +10785,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10799,7 +10803,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10817,7 +10821,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10839,7 +10843,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10861,7 +10865,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10883,7 +10887,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10905,7 +10909,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10927,7 +10931,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10950,7 +10954,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10972,7 +10976,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10994,7 +10998,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -11016,7 +11020,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -11038,7 +11042,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -11060,7 +11064,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11082,7 +11086,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11100,7 +11104,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11111,18 +11115,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11164,7 +11168,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11207,7 +11211,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11240,7 +11244,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11278,7 +11282,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11321,7 +11325,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11354,7 +11358,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11383,7 +11387,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11413,7 +11417,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11438,7 +11442,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11463,7 +11467,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11493,7 +11497,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11518,7 +11522,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11548,7 +11552,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11568,7 +11572,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11598,7 +11602,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11623,7 +11627,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11658,7 +11662,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11693,7 +11697,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11718,7 +11722,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11748,7 +11752,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11778,7 +11782,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11808,7 +11812,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11838,7 +11842,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11868,7 +11872,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11898,7 +11902,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11923,7 +11927,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11953,7 +11957,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -11983,7 +11987,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -12013,7 +12017,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -12048,7 +12052,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -12078,7 +12082,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12108,7 +12112,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12138,7 +12142,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12168,7 +12172,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12198,7 +12202,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12228,7 +12232,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12263,7 +12267,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12294,6 +12298,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-10-14 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46308</v>
+        <v>46309</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4108,7 +4108,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发3次</t>
+          <t>累计未发3次，迟发4次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-10-15 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46309</v>
+        <v>46310</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3940,7 +3940,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D37" s="71" t="n"/>
+      <c r="D37" s="71" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="E37" s="69" t="n"/>
       <c r="F37" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-10-17 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46310</v>
+        <v>46312</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4641,7 +4641,11 @@
           <t>是</t>
         </is>
       </c>
-      <c r="D62" s="68" t="n"/>
+      <c r="D62" s="68" t="inlineStr">
+        <is>
+          <t>迟发1次</t>
+        </is>
+      </c>
       <c r="E62" s="69" t="n"/>
       <c r="F62" s="63" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
report: update 2026-10-18 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46312</v>
+        <v>46313</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4112,7 +4112,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发4次</t>
+          <t>累计未发3次，迟发5次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发3次</t>
+          <t>累计未发4次，迟发3次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-10-22 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46313</v>
+        <v>46317</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="D38" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发1次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E38" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-10-23 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46317</v>
+        <v>46318</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4054,7 +4054,7 @@
       </c>
       <c r="D41" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E41" s="69" t="n"/>
@@ -4166,7 +4166,7 @@
       </c>
       <c r="D45" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发2次</t>
         </is>
       </c>
       <c r="E45" s="69" t="n"/>

</xml_diff>

<commit_message>
report: update 2026-10-24 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46318</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46319</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2812,7 +2812,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3083,7 +3083,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3175,7 +3175,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3217,7 +3217,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3263,7 +3263,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3300,7 +3300,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3331,7 +3331,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3611,7 +3611,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3642,7 +3642,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3855,7 +3855,7 @@
       </c>
       <c r="D34" s="71" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发1次</t>
+          <t>累计未发4次，迟发1次</t>
         </is>
       </c>
       <c r="E34" s="69" t="n"/>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4509,7 +4509,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4653,7 +4653,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4681,7 +4681,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4708,7 +4708,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="65" s="53">
       <c r="A65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -4730,7 +4730,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="66" s="53">
       <c r="A66" s="0" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4752,7 +4752,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="67" s="53">
       <c r="A67" s="0" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4769,204 +4769,204 @@
         </is>
       </c>
     </row>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4979,17 +4979,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -5012,7 +5012,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -5098,7 +5098,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5141,7 +5141,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5186,7 +5186,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5223,7 +5223,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5268,7 +5268,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5307,7 +5307,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5344,7 +5344,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5373,7 +5373,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5412,7 +5412,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5449,7 +5449,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5486,7 +5486,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5525,7 +5525,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5562,7 +5562,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5589,7 +5589,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5617,7 +5617,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5645,7 +5645,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5673,7 +5673,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5703,7 +5703,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5733,7 +5733,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5769,7 +5769,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5797,7 +5797,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5827,7 +5827,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5865,7 +5865,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5895,7 +5895,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5927,7 +5927,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5961,7 +5961,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5993,7 +5993,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6021,7 +6021,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6057,7 +6057,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6084,7 +6084,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6116,7 +6116,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6148,7 +6148,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6173,7 +6173,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6203,7 +6203,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6233,7 +6233,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6267,7 +6267,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6297,7 +6297,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6325,7 +6325,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6353,7 +6353,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6381,7 +6381,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6409,7 +6409,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6437,7 +6437,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6465,7 +6465,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6493,7 +6493,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6521,7 +6521,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6559,7 +6559,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6589,7 +6589,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6625,7 +6625,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6659,7 +6659,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6695,7 +6695,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6727,7 +6727,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7375,7 +7375,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7388,17 +7388,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7421,7 +7421,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7507,7 +7507,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7553,7 +7553,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7590,7 +7590,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7636,7 +7636,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7682,7 +7682,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7730,7 +7730,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7767,7 +7767,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7804,7 +7804,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7852,7 +7852,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7898,7 +7898,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7935,7 +7935,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7972,7 +7972,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8018,7 +8018,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8046,7 +8046,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8074,7 +8074,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8102,7 +8102,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8130,7 +8130,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8158,7 +8158,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8186,7 +8186,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8214,7 +8214,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8242,7 +8242,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8270,7 +8270,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8298,7 +8298,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8326,7 +8326,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8354,7 +8354,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8382,7 +8382,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8412,7 +8412,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8440,7 +8440,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8468,7 +8468,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8496,7 +8496,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8524,7 +8524,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8552,7 +8552,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8580,7 +8580,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8610,7 +8610,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8638,7 +8638,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8666,7 +8666,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8694,7 +8694,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8722,7 +8722,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8752,7 +8752,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8784,7 +8784,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8812,7 +8812,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8840,7 +8840,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8868,7 +8868,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8896,7 +8896,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8924,7 +8924,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8956,7 +8956,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8988,7 +8988,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9664,7 +9664,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9675,16 +9675,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9694,7 +9694,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9739,7 +9739,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9785,7 +9785,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9830,7 +9830,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9879,7 +9879,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9928,7 +9928,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9970,7 +9970,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10005,7 +10005,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10045,7 +10045,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10081,7 +10081,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10117,7 +10117,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10153,7 +10153,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10194,7 +10194,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10225,7 +10225,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10247,7 +10247,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10264,7 +10264,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10281,7 +10281,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10303,7 +10303,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10320,7 +10320,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10338,7 +10338,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10360,7 +10360,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10382,7 +10382,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10404,7 +10404,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10426,7 +10426,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10444,7 +10444,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10466,7 +10466,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10488,7 +10488,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10510,7 +10510,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10532,7 +10532,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10554,7 +10554,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10576,7 +10576,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10603,7 +10603,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10625,7 +10625,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10647,7 +10647,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10669,7 +10669,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10691,7 +10691,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10713,7 +10713,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10735,7 +10735,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10752,7 +10752,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10774,7 +10774,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10792,7 +10792,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10814,7 +10814,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10832,7 +10832,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10850,7 +10850,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10872,7 +10872,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10894,7 +10894,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10916,7 +10916,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10938,7 +10938,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10960,7 +10960,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10983,7 +10983,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -11005,7 +11005,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -11027,7 +11027,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -11049,7 +11049,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -11071,7 +11071,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -11093,7 +11093,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11115,7 +11115,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11133,7 +11133,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11144,18 +11144,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11197,7 +11197,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11240,7 +11240,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11273,7 +11273,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11311,7 +11311,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11354,7 +11354,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11387,7 +11387,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11416,7 +11416,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11446,7 +11446,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11471,7 +11471,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11496,7 +11496,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11526,7 +11526,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11551,7 +11551,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11581,7 +11581,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11601,7 +11601,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11631,7 +11631,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11656,7 +11656,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11691,7 +11691,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11726,7 +11726,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11751,7 +11751,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11781,7 +11781,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11811,7 +11811,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11841,7 +11841,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11871,7 +11871,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11901,7 +11901,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11931,7 +11931,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11956,7 +11956,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11986,7 +11986,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -12016,7 +12016,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -12046,7 +12046,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -12081,7 +12081,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -12111,7 +12111,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12141,7 +12141,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12171,7 +12171,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12201,7 +12201,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12231,7 +12231,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12261,7 +12261,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12296,7 +12296,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12327,6 +12327,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-10-25 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46319</v>
+        <v>46320</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3523,7 +3523,7 @@
       </c>
       <c r="D22" s="70" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E22" s="69" t="n"/>
@@ -4249,7 +4249,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>累计未发1次，迟发2次</t>
+          <t>累计未发2次，迟发2次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4766,6 +4766,11 @@
       <c r="C67" s="0" t="inlineStr">
         <is>
           <t>是</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
report: update 2026-10-27 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46320</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46322</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2812,7 +2812,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3083,7 +3083,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3175,7 +3175,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3217,7 +3217,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3263,7 +3263,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3300,7 +3300,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3331,7 +3331,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3611,7 +3611,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3642,7 +3642,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3714,7 +3714,7 @@
       </c>
       <c r="D29" s="70" t="inlineStr">
         <is>
-          <t>迟发1次</t>
+          <t>累计未发1次，迟发1次</t>
         </is>
       </c>
       <c r="E29" s="69" t="n"/>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发4次，迟发3次</t>
+          <t>累计未发5次，迟发3次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4509,7 +4509,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4653,7 +4653,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4681,7 +4681,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4708,7 +4708,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="65" s="53">
       <c r="A65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -4730,7 +4730,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="66" s="53">
       <c r="A66" s="0" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4746,13 +4746,18 @@
           <t>是</t>
         </is>
       </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>累计未发1次</t>
+        </is>
+      </c>
       <c r="F66" s="0" t="inlineStr">
         <is>
           <t>华北分公司</t>
         </is>
       </c>
     </row>
-    <row r="67" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="67" s="53">
       <c r="A67" s="0" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4770,208 +4775,208 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>累计未发1次</t>
-        </is>
-      </c>
-    </row>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+          <t>累计未发2次</t>
+        </is>
+      </c>
+    </row>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4984,17 +4989,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -5017,7 +5022,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -5103,7 +5108,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5146,7 +5151,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5191,7 +5196,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5228,7 +5233,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5273,7 +5278,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5312,7 +5317,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5349,7 +5354,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5378,7 +5383,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5417,7 +5422,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5454,7 +5459,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5491,7 +5496,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5530,7 +5535,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5567,7 +5572,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5594,7 +5599,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5622,7 +5627,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5650,7 +5655,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5678,7 +5683,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5708,7 +5713,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5738,7 +5743,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5774,7 +5779,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5802,7 +5807,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5832,7 +5837,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5870,7 +5875,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5900,7 +5905,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5932,7 +5937,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5966,7 +5971,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5998,7 +6003,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6026,7 +6031,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6062,7 +6067,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6089,7 +6094,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6121,7 +6126,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6153,7 +6158,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6178,7 +6183,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6208,7 +6213,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6238,7 +6243,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6272,7 +6277,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6302,7 +6307,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6330,7 +6335,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6358,7 +6363,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6386,7 +6391,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6414,7 +6419,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6442,7 +6447,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6470,7 +6475,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6498,7 +6503,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6526,7 +6531,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6564,7 +6569,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6594,7 +6599,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6630,7 +6635,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6664,7 +6669,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6700,7 +6705,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6732,7 +6737,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7380,7 +7385,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7393,17 +7398,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7426,7 +7431,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7512,7 +7517,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7558,7 +7563,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7595,7 +7600,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7641,7 +7646,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7687,7 +7692,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7735,7 +7740,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7772,7 +7777,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7809,7 +7814,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7857,7 +7862,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7903,7 +7908,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7940,7 +7945,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7977,7 +7982,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8023,7 +8028,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8051,7 +8056,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8079,7 +8084,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8107,7 +8112,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8135,7 +8140,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8163,7 +8168,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8191,7 +8196,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8219,7 +8224,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8247,7 +8252,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8275,7 +8280,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8303,7 +8308,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8331,7 +8336,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8359,7 +8364,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8387,7 +8392,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8417,7 +8422,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8445,7 +8450,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8473,7 +8478,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8501,7 +8506,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8529,7 +8534,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8557,7 +8562,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8585,7 +8590,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8615,7 +8620,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8643,7 +8648,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8671,7 +8676,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8699,7 +8704,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8727,7 +8732,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8757,7 +8762,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8789,7 +8794,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8817,7 +8822,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8845,7 +8850,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8873,7 +8878,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8901,7 +8906,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8929,7 +8934,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8961,7 +8966,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8993,7 +8998,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9669,7 +9674,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9680,16 +9685,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9699,7 +9704,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9744,7 +9749,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9790,7 +9795,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9835,7 +9840,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9884,7 +9889,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9933,7 +9938,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9975,7 +9980,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10010,7 +10015,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10050,7 +10055,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10086,7 +10091,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10122,7 +10127,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10158,7 +10163,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10199,7 +10204,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10230,7 +10235,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10252,7 +10257,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10269,7 +10274,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10286,7 +10291,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10308,7 +10313,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10325,7 +10330,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10343,7 +10348,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10365,7 +10370,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10387,7 +10392,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10409,7 +10414,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10431,7 +10436,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10449,7 +10454,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10471,7 +10476,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10493,7 +10498,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10515,7 +10520,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10537,7 +10542,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10559,7 +10564,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10581,7 +10586,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10608,7 +10613,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10630,7 +10635,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10652,7 +10657,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10674,7 +10679,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10696,7 +10701,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10718,7 +10723,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10740,7 +10745,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10757,7 +10762,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10779,7 +10784,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10797,7 +10802,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10819,7 +10824,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10837,7 +10842,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10855,7 +10860,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10877,7 +10882,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10899,7 +10904,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10921,7 +10926,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10943,7 +10948,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10965,7 +10970,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10988,7 +10993,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -11010,7 +11015,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -11032,7 +11037,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -11054,7 +11059,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -11076,7 +11081,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -11098,7 +11103,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11120,7 +11125,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11138,7 +11143,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11149,18 +11154,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11202,7 +11207,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11245,7 +11250,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11278,7 +11283,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11316,7 +11321,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11359,7 +11364,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11392,7 +11397,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11421,7 +11426,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11451,7 +11456,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11476,7 +11481,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11501,7 +11506,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11531,7 +11536,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11556,7 +11561,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11586,7 +11591,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11606,7 +11611,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11636,7 +11641,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11661,7 +11666,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11696,7 +11701,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11731,7 +11736,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11756,7 +11761,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11786,7 +11791,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11816,7 +11821,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11846,7 +11851,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11876,7 +11881,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11906,7 +11911,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11936,7 +11941,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11961,7 +11966,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -11991,7 +11996,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -12021,7 +12026,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -12051,7 +12056,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -12086,7 +12091,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -12116,7 +12121,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12146,7 +12151,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12176,7 +12181,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12206,7 +12211,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12236,7 +12241,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12266,7 +12271,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12301,7 +12306,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12332,6 +12337,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-10-29 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="500" windowWidth="27040" windowHeight="16400" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
+    <workbookView activeTab="1" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible" windowHeight="16400" windowWidth="27040" xWindow="0" yWindow="500"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
+    <sheet name="2025年日报" sheetId="1" state="hidden" r:id="rId1"/>
+    <sheet name="2026年日报" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="2025月报" sheetId="3" state="hidden" r:id="rId3"/>
+    <sheet name="月报(2026)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="2026年日报 (2026-4-9存档)" sheetId="5" state="hidden" r:id="rId5"/>
+    <sheet name="旧表" sheetId="6" state="hidden" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'2026年日报'!$A$2:$F$61</definedName>
+    <definedName hidden="1" localSheetId="1" name="_xlnm._FilterDatabase">'2026年日报'!$A$2:$F$61</definedName>
   </definedNames>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
 </workbook>
@@ -449,257 +449,257 @@
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="7" applyAlignment="1">
+    <xf applyAlignment="1" borderId="7" fillId="7" fontId="0" numFmtId="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
   <cellXfs count="83">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="0" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="3" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="7" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="5" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="2" fillId="2" fontId="8" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="5" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="6" fillId="4" fontId="6" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="5" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="10" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="11" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="12" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="11" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="16" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="13" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="13" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="17" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="17" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="15" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="15" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="0" fillId="0" fontId="0" numFmtId="14" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="4" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="14" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="18" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="18" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="16" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="3" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="9" fillId="3" fontId="2" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="7" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="0" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="10" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="12" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="13" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="9" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="2" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="6" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="6" fontId="14" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="20" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="20" fillId="7" fontId="17" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="7" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="19" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="19" fillId="2" fontId="4" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="8" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf applyAlignment="1" borderId="8" fillId="2" fontId="1" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="1" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf borderId="9" fillId="0" fontId="0" numFmtId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="常规" xfId="0" builtinId="0"/>
+    <cellStyle builtinId="0" name="常规" xfId="0"/>
   </cellStyles>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <tableStyles count="0" defaultPivotStyle="PivotStyleLight16" defaultTableStyle="TableStyleMedium2"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="00000000"/>
@@ -1073,16 +1073,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -1127,7 +1127,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1181,7 +1181,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1235,7 +1235,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1284,7 +1284,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1338,7 +1338,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -1387,7 +1387,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1432,7 +1432,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1472,7 +1472,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -1517,7 +1517,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1557,7 +1557,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1597,7 +1597,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1642,7 +1642,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1682,7 +1682,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -1704,7 +1704,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1721,7 +1721,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1738,7 +1738,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -1760,7 +1760,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1804,7 +1804,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1826,7 +1826,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1849,7 +1849,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -1871,7 +1871,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1893,7 +1893,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1920,7 +1920,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -1942,7 +1942,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1969,7 +1969,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -1991,7 +1991,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -2013,7 +2013,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2035,7 +2035,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2057,7 +2057,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2084,7 +2084,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2106,7 +2106,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -2128,7 +2128,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2155,7 +2155,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2177,7 +2177,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2204,7 +2204,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2226,7 +2226,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2265,7 +2265,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2283,7 +2283,7 @@
       </c>
       <c r="D40" s="46" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2305,7 +2305,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -2332,7 +2332,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2354,7 +2354,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2376,7 +2376,7 @@
         </is>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2398,7 +2398,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -2420,7 +2420,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2447,7 +2447,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="D48" s="51" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2487,7 +2487,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2509,7 +2509,7 @@
         </is>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2558,7 +2558,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2585,7 +2585,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -2608,7 +2608,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -2619,26 +2619,26 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:O67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46322</v>
-      </c>
-    </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+        <v>46324</v>
+      </c>
+    </row>
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="61" t="inlineStr">
         <is>
           <t>区域</t>
@@ -2688,7 +2688,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2748,7 +2748,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2812,7 +2812,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2876,7 +2876,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2931,7 +2931,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -2986,7 +2986,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3032,7 +3032,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3083,7 +3083,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="61" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -3129,7 +3129,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3175,7 +3175,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3217,7 +3217,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3263,7 +3263,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3300,7 +3300,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="15" s="78">
       <c r="A15" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3331,7 +3331,7 @@
       <c r="H15" s="23" t="n"/>
       <c r="J15" s="67" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3368,7 +3368,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3386,7 +3386,7 @@
       </c>
       <c r="D17" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发2次，迟发1次</t>
         </is>
       </c>
       <c r="E17" s="69" t="n"/>
@@ -3397,7 +3397,7 @@
       </c>
       <c r="G17" s="67" t="n"/>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3422,7 +3422,7 @@
       </c>
       <c r="G18" s="67" t="n"/>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="61" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="G19" s="67" t="n"/>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3476,7 +3476,7 @@
       </c>
       <c r="G20" s="67" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3505,7 +3505,7 @@
       </c>
       <c r="G21" s="67" t="n"/>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3534,7 +3534,7 @@
       </c>
       <c r="G22" s="67" t="n"/>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3559,7 +3559,7 @@
       </c>
       <c r="G23" s="67" t="n"/>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3584,7 +3584,7 @@
       </c>
       <c r="G24" s="67" t="n"/>
     </row>
-    <row r="25" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="25" s="78">
       <c r="A25" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3611,7 +3611,7 @@
       <c r="H25" s="67" t="n"/>
       <c r="J25" s="67" t="n"/>
     </row>
-    <row r="26" ht="16.5" customFormat="1" customHeight="1" s="78">
+    <row customFormat="1" customHeight="1" ht="16.5" r="26" s="78">
       <c r="A26" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3642,7 +3642,7 @@
       <c r="H26" s="67" t="n"/>
       <c r="J26" s="67" t="n"/>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3671,7 +3671,7 @@
       </c>
       <c r="G27" s="67" t="n"/>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3696,7 +3696,7 @@
       </c>
       <c r="G28" s="67" t="n"/>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="G29" s="67" t="n"/>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3754,7 +3754,7 @@
       </c>
       <c r="G30" s="67" t="n"/>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3783,7 +3783,7 @@
       </c>
       <c r="G31" s="67" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="61" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -3808,7 +3808,7 @@
       </c>
       <c r="G32" s="67" t="n"/>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3837,7 +3837,7 @@
       </c>
       <c r="G33" s="67" t="n"/>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3866,7 +3866,7 @@
       </c>
       <c r="G34" s="67" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="G35" s="67" t="n"/>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3924,7 +3924,7 @@
       </c>
       <c r="G36" s="67" t="n"/>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="61" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="G37" s="67" t="n"/>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -3982,7 +3982,7 @@
       </c>
       <c r="G38" s="67" t="n"/>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="G39" s="67" t="n"/>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4036,7 +4036,7 @@
       </c>
       <c r="G40" s="67" t="n"/>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4065,7 +4065,7 @@
       </c>
       <c r="G41" s="67" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4094,7 +4094,7 @@
       </c>
       <c r="G42" s="67" t="n"/>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4112,7 +4112,7 @@
       </c>
       <c r="D43" s="68" t="inlineStr">
         <is>
-          <t>累计未发3次，迟发5次</t>
+          <t>累计未发4次，迟发5次</t>
         </is>
       </c>
       <c r="E43" s="69" t="n"/>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="G43" s="67" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4148,7 +4148,7 @@
       </c>
       <c r="G44" s="67" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4177,7 +4177,7 @@
       </c>
       <c r="G45" s="67" t="n"/>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4202,7 +4202,7 @@
       </c>
       <c r="G46" s="67" t="n"/>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4231,7 +4231,7 @@
       </c>
       <c r="G47" s="67" t="n"/>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4260,7 +4260,7 @@
       </c>
       <c r="G48" s="67" t="n"/>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4289,7 +4289,7 @@
       </c>
       <c r="G49" s="67" t="n"/>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4314,7 +4314,7 @@
       </c>
       <c r="G50" s="67" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4343,7 +4343,7 @@
       </c>
       <c r="G51" s="67" t="n"/>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="61" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4368,7 +4368,7 @@
       </c>
       <c r="G52" s="67" t="n"/>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="72" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4397,7 +4397,7 @@
       </c>
       <c r="G53" s="67" t="n"/>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="58" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4426,7 +4426,7 @@
       </c>
       <c r="G54" s="67" t="n"/>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="58" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4455,7 +4455,7 @@
       </c>
       <c r="G55" s="67" t="n"/>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4480,7 +4480,7 @@
       </c>
       <c r="G56" s="67" t="n"/>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="58" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4509,7 +4509,7 @@
       </c>
       <c r="G57" s="67" t="n"/>
     </row>
-    <row r="58" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="58" s="53">
       <c r="A58" s="60" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4538,7 +4538,7 @@
       </c>
       <c r="G58" s="67" t="n"/>
     </row>
-    <row r="59" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="59" s="53">
       <c r="A59" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4556,7 +4556,7 @@
       </c>
       <c r="D59" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发3次，迟发2次</t>
         </is>
       </c>
       <c r="E59" s="69" t="n"/>
@@ -4567,7 +4567,7 @@
       </c>
       <c r="G59" s="67" t="n"/>
     </row>
-    <row r="60" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="60" s="53">
       <c r="A60" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4596,7 +4596,7 @@
       </c>
       <c r="G60" s="67" t="n"/>
     </row>
-    <row r="61" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="61" s="53">
       <c r="A61" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4625,7 +4625,7 @@
       </c>
       <c r="G61" s="67" t="n"/>
     </row>
-    <row r="62" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="62" s="53">
       <c r="A62" s="60" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4653,7 +4653,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="63" s="53">
       <c r="A63" s="60" t="inlineStr">
         <is>
           <t>粤东区</t>
@@ -4681,7 +4681,7 @@
         </is>
       </c>
     </row>
-    <row r="64" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="64" s="53">
       <c r="A64" s="0" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -4708,7 +4708,7 @@
         </is>
       </c>
     </row>
-    <row r="65" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="65" s="53">
       <c r="A65" s="0" t="inlineStr">
         <is>
           <t>华东分公司</t>
@@ -4730,7 +4730,7 @@
         </is>
       </c>
     </row>
-    <row r="66" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="66" s="53">
       <c r="A66" s="0" t="inlineStr">
         <is>
           <t>粤西区</t>
@@ -4757,7 +4757,7 @@
         </is>
       </c>
     </row>
-    <row r="67" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="67" s="53">
       <c r="A67" s="0" t="inlineStr">
         <is>
           <t>华北分公司</t>
@@ -4778,210 +4778,210 @@
           <t>累计未发2次</t>
         </is>
       </c>
-      <c r="F67" t="inlineStr">
+      <c r="F67" s="0" t="inlineStr">
         <is>
           <t>华北分公司</t>
         </is>
       </c>
     </row>
-    <row r="68" ht="16" customHeight="1" s="53"/>
-    <row r="69" ht="16" customHeight="1" s="53"/>
-    <row r="70" ht="16" customHeight="1" s="53"/>
-    <row r="71" ht="16" customHeight="1" s="53"/>
-    <row r="72" ht="16" customHeight="1" s="53"/>
-    <row r="73" ht="16" customHeight="1" s="53"/>
-    <row r="74" ht="16" customHeight="1" s="53"/>
-    <row r="75" ht="16" customHeight="1" s="53"/>
-    <row r="76" ht="16" customHeight="1" s="53"/>
-    <row r="77" ht="16" customHeight="1" s="53"/>
-    <row r="78" ht="16" customHeight="1" s="53"/>
-    <row r="79" ht="16" customHeight="1" s="53"/>
-    <row r="80" ht="16" customHeight="1" s="53"/>
-    <row r="81" ht="16" customHeight="1" s="53"/>
-    <row r="82" ht="16" customHeight="1" s="53"/>
-    <row r="83" ht="16" customHeight="1" s="53"/>
-    <row r="84" ht="16" customHeight="1" s="53"/>
-    <row r="85" ht="16" customHeight="1" s="53"/>
-    <row r="86" ht="16" customHeight="1" s="53"/>
-    <row r="87" ht="16" customHeight="1" s="53"/>
-    <row r="88" ht="16" customHeight="1" s="53"/>
-    <row r="89" ht="16" customHeight="1" s="53"/>
-    <row r="90" ht="16" customHeight="1" s="53"/>
-    <row r="91" ht="16" customHeight="1" s="53"/>
-    <row r="92" ht="16" customHeight="1" s="53"/>
-    <row r="93" ht="16" customHeight="1" s="53"/>
-    <row r="94" ht="16" customHeight="1" s="53"/>
-    <row r="95" ht="16" customHeight="1" s="53"/>
-    <row r="96" ht="16" customHeight="1" s="53"/>
-    <row r="97" ht="16" customHeight="1" s="53"/>
-    <row r="98" ht="16" customHeight="1" s="53"/>
-    <row r="99" ht="16" customHeight="1" s="53"/>
-    <row r="100" ht="16" customHeight="1" s="53"/>
-    <row r="101" ht="16" customHeight="1" s="53"/>
-    <row r="102" ht="16" customHeight="1" s="53"/>
-    <row r="103" ht="16" customHeight="1" s="53"/>
-    <row r="104" ht="16" customHeight="1" s="53"/>
-    <row r="105" ht="16" customHeight="1" s="53"/>
-    <row r="106" ht="16" customHeight="1" s="53"/>
-    <row r="107" ht="16" customHeight="1" s="53"/>
-    <row r="108" ht="16" customHeight="1" s="53"/>
-    <row r="109" ht="16" customHeight="1" s="53"/>
-    <row r="110" ht="16" customHeight="1" s="53"/>
-    <row r="111" ht="16" customHeight="1" s="53"/>
-    <row r="112" ht="16" customHeight="1" s="53"/>
-    <row r="113" ht="16" customHeight="1" s="53"/>
-    <row r="114" ht="16" customHeight="1" s="53"/>
-    <row r="115" ht="16" customHeight="1" s="53"/>
-    <row r="116" ht="16" customHeight="1" s="53"/>
-    <row r="117" ht="16" customHeight="1" s="53"/>
-    <row r="118" ht="16" customHeight="1" s="53"/>
-    <row r="119" ht="16" customHeight="1" s="53"/>
-    <row r="120" ht="16" customHeight="1" s="53"/>
-    <row r="121" ht="16" customHeight="1" s="53"/>
-    <row r="122" ht="16" customHeight="1" s="53"/>
-    <row r="123" ht="16" customHeight="1" s="53"/>
-    <row r="124" ht="16" customHeight="1" s="53"/>
-    <row r="125" ht="16" customHeight="1" s="53"/>
-    <row r="126" ht="16" customHeight="1" s="53"/>
-    <row r="127" ht="16" customHeight="1" s="53"/>
-    <row r="128" ht="16" customHeight="1" s="53"/>
-    <row r="129" ht="16" customHeight="1" s="53"/>
-    <row r="130" ht="16" customHeight="1" s="53"/>
-    <row r="131" ht="16" customHeight="1" s="53"/>
-    <row r="132" ht="16" customHeight="1" s="53"/>
-    <row r="133" ht="16" customHeight="1" s="53"/>
-    <row r="134" ht="16" customHeight="1" s="53"/>
-    <row r="135" ht="16" customHeight="1" s="53"/>
-    <row r="136" ht="16" customHeight="1" s="53"/>
-    <row r="137" ht="16" customHeight="1" s="53"/>
-    <row r="138" ht="16" customHeight="1" s="53"/>
-    <row r="139" ht="16" customHeight="1" s="53"/>
-    <row r="140" ht="16" customHeight="1" s="53"/>
-    <row r="141" ht="16" customHeight="1" s="53"/>
-    <row r="142" ht="16" customHeight="1" s="53"/>
-    <row r="143" ht="16" customHeight="1" s="53"/>
-    <row r="144" ht="16" customHeight="1" s="53"/>
-    <row r="145" ht="16" customHeight="1" s="53"/>
-    <row r="146" ht="16" customHeight="1" s="53"/>
-    <row r="147" ht="16" customHeight="1" s="53"/>
-    <row r="148" ht="16" customHeight="1" s="53"/>
-    <row r="149" ht="16" customHeight="1" s="53"/>
-    <row r="150" ht="16" customHeight="1" s="53"/>
-    <row r="151" ht="16" customHeight="1" s="53"/>
-    <row r="152" ht="16" customHeight="1" s="53"/>
-    <row r="153" ht="16" customHeight="1" s="53"/>
-    <row r="154" ht="16" customHeight="1" s="53"/>
-    <row r="155" ht="16" customHeight="1" s="53"/>
-    <row r="156" ht="16" customHeight="1" s="53"/>
-    <row r="157" ht="16" customHeight="1" s="53"/>
-    <row r="158" ht="16" customHeight="1" s="53"/>
-    <row r="159" ht="16" customHeight="1" s="53"/>
-    <row r="160" ht="16" customHeight="1" s="53"/>
-    <row r="161" ht="16" customHeight="1" s="53"/>
-    <row r="162" ht="16" customHeight="1" s="53"/>
-    <row r="163" ht="16" customHeight="1" s="53"/>
-    <row r="164" ht="16" customHeight="1" s="53"/>
-    <row r="165" ht="16" customHeight="1" s="53"/>
-    <row r="166" ht="16" customHeight="1" s="53"/>
-    <row r="167" ht="16" customHeight="1" s="53"/>
-    <row r="168" ht="16" customHeight="1" s="53"/>
-    <row r="169" ht="16" customHeight="1" s="53"/>
-    <row r="170" ht="16" customHeight="1" s="53"/>
-    <row r="171" ht="16" customHeight="1" s="53"/>
-    <row r="172" ht="16" customHeight="1" s="53"/>
-    <row r="173" ht="16" customHeight="1" s="53"/>
-    <row r="174" ht="16" customHeight="1" s="53"/>
-    <row r="175" ht="16" customHeight="1" s="53"/>
-    <row r="176" ht="16" customHeight="1" s="53"/>
-    <row r="177" ht="16" customHeight="1" s="53"/>
-    <row r="178" ht="16" customHeight="1" s="53"/>
-    <row r="179" ht="16" customHeight="1" s="53"/>
-    <row r="180" ht="16" customHeight="1" s="53"/>
-    <row r="181" ht="16" customHeight="1" s="53"/>
-    <row r="182" ht="16" customHeight="1" s="53"/>
-    <row r="183" ht="16" customHeight="1" s="53"/>
-    <row r="184" ht="16" customHeight="1" s="53"/>
-    <row r="185" ht="16" customHeight="1" s="53"/>
-    <row r="186" ht="16" customHeight="1" s="53"/>
-    <row r="187" ht="16" customHeight="1" s="53"/>
-    <row r="188" ht="16" customHeight="1" s="53"/>
-    <row r="189" ht="16" customHeight="1" s="53"/>
-    <row r="190" ht="16" customHeight="1" s="53"/>
-    <row r="191" ht="16" customHeight="1" s="53"/>
-    <row r="192" ht="16" customHeight="1" s="53"/>
-    <row r="193" ht="16" customHeight="1" s="53"/>
-    <row r="194" ht="16" customHeight="1" s="53"/>
-    <row r="195" ht="16" customHeight="1" s="53"/>
-    <row r="196" ht="16" customHeight="1" s="53"/>
-    <row r="197" ht="16" customHeight="1" s="53"/>
-    <row r="198" ht="16" customHeight="1" s="53"/>
-    <row r="199" ht="16" customHeight="1" s="53"/>
-    <row r="200" ht="16" customHeight="1" s="53"/>
-    <row r="201" ht="16" customHeight="1" s="53"/>
-    <row r="202" ht="16" customHeight="1" s="53"/>
-    <row r="203" ht="16" customHeight="1" s="53"/>
-    <row r="204" ht="16" customHeight="1" s="53"/>
-    <row r="205" ht="16" customHeight="1" s="53"/>
-    <row r="206" ht="16" customHeight="1" s="53"/>
-    <row r="207" ht="16" customHeight="1" s="53"/>
-    <row r="208" ht="16" customHeight="1" s="53"/>
-    <row r="209" ht="16" customHeight="1" s="53"/>
-    <row r="210" ht="16" customHeight="1" s="53"/>
-    <row r="211" ht="16" customHeight="1" s="53"/>
-    <row r="212" ht="16" customHeight="1" s="53"/>
-    <row r="213" ht="16" customHeight="1" s="53"/>
-    <row r="214" ht="16" customHeight="1" s="53"/>
-    <row r="215" ht="16" customHeight="1" s="53"/>
-    <row r="216" ht="16" customHeight="1" s="53"/>
-    <row r="217" ht="16" customHeight="1" s="53"/>
-    <row r="218" ht="16" customHeight="1" s="53"/>
-    <row r="219" ht="16" customHeight="1" s="53"/>
-    <row r="220" ht="16" customHeight="1" s="53"/>
-    <row r="221" ht="16" customHeight="1" s="53"/>
-    <row r="222" ht="16" customHeight="1" s="53"/>
-    <row r="223" ht="16" customHeight="1" s="53"/>
-    <row r="224" ht="16" customHeight="1" s="53"/>
-    <row r="225" ht="16" customHeight="1" s="53"/>
-    <row r="226" ht="16" customHeight="1" s="53"/>
-    <row r="227" ht="16" customHeight="1" s="53"/>
-    <row r="228" ht="16" customHeight="1" s="53"/>
-    <row r="229" ht="16" customHeight="1" s="53"/>
-    <row r="230" ht="16" customHeight="1" s="53"/>
-    <row r="231" ht="16" customHeight="1" s="53"/>
-    <row r="232" ht="16" customHeight="1" s="53"/>
-    <row r="233" ht="16" customHeight="1" s="53"/>
-    <row r="234" ht="16" customHeight="1" s="53"/>
-    <row r="235" ht="16" customHeight="1" s="53"/>
-    <row r="236" ht="16" customHeight="1" s="53"/>
-    <row r="237" ht="16" customHeight="1" s="53"/>
-    <row r="238" ht="16" customHeight="1" s="53"/>
-    <row r="239" ht="16" customHeight="1" s="53"/>
-    <row r="240" ht="16" customHeight="1" s="53"/>
-    <row r="241" ht="16" customHeight="1" s="53"/>
-    <row r="242" ht="16" customHeight="1" s="53"/>
-    <row r="243" ht="16" customHeight="1" s="53"/>
-    <row r="244" ht="16" customHeight="1" s="53"/>
-    <row r="245" ht="16" customHeight="1" s="53"/>
-    <row r="246" ht="16" customHeight="1" s="53"/>
-    <row r="247" ht="16" customHeight="1" s="53"/>
-    <row r="248" ht="16" customHeight="1" s="53"/>
-    <row r="249" ht="16" customHeight="1" s="53"/>
-    <row r="250" ht="16" customHeight="1" s="53"/>
-    <row r="251" ht="16" customHeight="1" s="53"/>
-    <row r="252" ht="16" customHeight="1" s="53"/>
-    <row r="253" ht="16" customHeight="1" s="53"/>
-    <row r="254" ht="16" customHeight="1" s="53"/>
-    <row r="255" ht="16" customHeight="1" s="53"/>
-    <row r="256" ht="16" customHeight="1" s="53"/>
-    <row r="257" ht="16" customHeight="1" s="53"/>
-    <row r="258" ht="16" customHeight="1" s="53"/>
-    <row r="259" ht="16" customHeight="1" s="53"/>
-    <row r="260" ht="16" customHeight="1" s="53"/>
-    <row r="261" ht="16" customHeight="1" s="53"/>
-    <row r="262" ht="16" customHeight="1" s="53"/>
+    <row customHeight="1" ht="16" r="68" s="53"/>
+    <row customHeight="1" ht="16" r="69" s="53"/>
+    <row customHeight="1" ht="16" r="70" s="53"/>
+    <row customHeight="1" ht="16" r="71" s="53"/>
+    <row customHeight="1" ht="16" r="72" s="53"/>
+    <row customHeight="1" ht="16" r="73" s="53"/>
+    <row customHeight="1" ht="16" r="74" s="53"/>
+    <row customHeight="1" ht="16" r="75" s="53"/>
+    <row customHeight="1" ht="16" r="76" s="53"/>
+    <row customHeight="1" ht="16" r="77" s="53"/>
+    <row customHeight="1" ht="16" r="78" s="53"/>
+    <row customHeight="1" ht="16" r="79" s="53"/>
+    <row customHeight="1" ht="16" r="80" s="53"/>
+    <row customHeight="1" ht="16" r="81" s="53"/>
+    <row customHeight="1" ht="16" r="82" s="53"/>
+    <row customHeight="1" ht="16" r="83" s="53"/>
+    <row customHeight="1" ht="16" r="84" s="53"/>
+    <row customHeight="1" ht="16" r="85" s="53"/>
+    <row customHeight="1" ht="16" r="86" s="53"/>
+    <row customHeight="1" ht="16" r="87" s="53"/>
+    <row customHeight="1" ht="16" r="88" s="53"/>
+    <row customHeight="1" ht="16" r="89" s="53"/>
+    <row customHeight="1" ht="16" r="90" s="53"/>
+    <row customHeight="1" ht="16" r="91" s="53"/>
+    <row customHeight="1" ht="16" r="92" s="53"/>
+    <row customHeight="1" ht="16" r="93" s="53"/>
+    <row customHeight="1" ht="16" r="94" s="53"/>
+    <row customHeight="1" ht="16" r="95" s="53"/>
+    <row customHeight="1" ht="16" r="96" s="53"/>
+    <row customHeight="1" ht="16" r="97" s="53"/>
+    <row customHeight="1" ht="16" r="98" s="53"/>
+    <row customHeight="1" ht="16" r="99" s="53"/>
+    <row customHeight="1" ht="16" r="100" s="53"/>
+    <row customHeight="1" ht="16" r="101" s="53"/>
+    <row customHeight="1" ht="16" r="102" s="53"/>
+    <row customHeight="1" ht="16" r="103" s="53"/>
+    <row customHeight="1" ht="16" r="104" s="53"/>
+    <row customHeight="1" ht="16" r="105" s="53"/>
+    <row customHeight="1" ht="16" r="106" s="53"/>
+    <row customHeight="1" ht="16" r="107" s="53"/>
+    <row customHeight="1" ht="16" r="108" s="53"/>
+    <row customHeight="1" ht="16" r="109" s="53"/>
+    <row customHeight="1" ht="16" r="110" s="53"/>
+    <row customHeight="1" ht="16" r="111" s="53"/>
+    <row customHeight="1" ht="16" r="112" s="53"/>
+    <row customHeight="1" ht="16" r="113" s="53"/>
+    <row customHeight="1" ht="16" r="114" s="53"/>
+    <row customHeight="1" ht="16" r="115" s="53"/>
+    <row customHeight="1" ht="16" r="116" s="53"/>
+    <row customHeight="1" ht="16" r="117" s="53"/>
+    <row customHeight="1" ht="16" r="118" s="53"/>
+    <row customHeight="1" ht="16" r="119" s="53"/>
+    <row customHeight="1" ht="16" r="120" s="53"/>
+    <row customHeight="1" ht="16" r="121" s="53"/>
+    <row customHeight="1" ht="16" r="122" s="53"/>
+    <row customHeight="1" ht="16" r="123" s="53"/>
+    <row customHeight="1" ht="16" r="124" s="53"/>
+    <row customHeight="1" ht="16" r="125" s="53"/>
+    <row customHeight="1" ht="16" r="126" s="53"/>
+    <row customHeight="1" ht="16" r="127" s="53"/>
+    <row customHeight="1" ht="16" r="128" s="53"/>
+    <row customHeight="1" ht="16" r="129" s="53"/>
+    <row customHeight="1" ht="16" r="130" s="53"/>
+    <row customHeight="1" ht="16" r="131" s="53"/>
+    <row customHeight="1" ht="16" r="132" s="53"/>
+    <row customHeight="1" ht="16" r="133" s="53"/>
+    <row customHeight="1" ht="16" r="134" s="53"/>
+    <row customHeight="1" ht="16" r="135" s="53"/>
+    <row customHeight="1" ht="16" r="136" s="53"/>
+    <row customHeight="1" ht="16" r="137" s="53"/>
+    <row customHeight="1" ht="16" r="138" s="53"/>
+    <row customHeight="1" ht="16" r="139" s="53"/>
+    <row customHeight="1" ht="16" r="140" s="53"/>
+    <row customHeight="1" ht="16" r="141" s="53"/>
+    <row customHeight="1" ht="16" r="142" s="53"/>
+    <row customHeight="1" ht="16" r="143" s="53"/>
+    <row customHeight="1" ht="16" r="144" s="53"/>
+    <row customHeight="1" ht="16" r="145" s="53"/>
+    <row customHeight="1" ht="16" r="146" s="53"/>
+    <row customHeight="1" ht="16" r="147" s="53"/>
+    <row customHeight="1" ht="16" r="148" s="53"/>
+    <row customHeight="1" ht="16" r="149" s="53"/>
+    <row customHeight="1" ht="16" r="150" s="53"/>
+    <row customHeight="1" ht="16" r="151" s="53"/>
+    <row customHeight="1" ht="16" r="152" s="53"/>
+    <row customHeight="1" ht="16" r="153" s="53"/>
+    <row customHeight="1" ht="16" r="154" s="53"/>
+    <row customHeight="1" ht="16" r="155" s="53"/>
+    <row customHeight="1" ht="16" r="156" s="53"/>
+    <row customHeight="1" ht="16" r="157" s="53"/>
+    <row customHeight="1" ht="16" r="158" s="53"/>
+    <row customHeight="1" ht="16" r="159" s="53"/>
+    <row customHeight="1" ht="16" r="160" s="53"/>
+    <row customHeight="1" ht="16" r="161" s="53"/>
+    <row customHeight="1" ht="16" r="162" s="53"/>
+    <row customHeight="1" ht="16" r="163" s="53"/>
+    <row customHeight="1" ht="16" r="164" s="53"/>
+    <row customHeight="1" ht="16" r="165" s="53"/>
+    <row customHeight="1" ht="16" r="166" s="53"/>
+    <row customHeight="1" ht="16" r="167" s="53"/>
+    <row customHeight="1" ht="16" r="168" s="53"/>
+    <row customHeight="1" ht="16" r="169" s="53"/>
+    <row customHeight="1" ht="16" r="170" s="53"/>
+    <row customHeight="1" ht="16" r="171" s="53"/>
+    <row customHeight="1" ht="16" r="172" s="53"/>
+    <row customHeight="1" ht="16" r="173" s="53"/>
+    <row customHeight="1" ht="16" r="174" s="53"/>
+    <row customHeight="1" ht="16" r="175" s="53"/>
+    <row customHeight="1" ht="16" r="176" s="53"/>
+    <row customHeight="1" ht="16" r="177" s="53"/>
+    <row customHeight="1" ht="16" r="178" s="53"/>
+    <row customHeight="1" ht="16" r="179" s="53"/>
+    <row customHeight="1" ht="16" r="180" s="53"/>
+    <row customHeight="1" ht="16" r="181" s="53"/>
+    <row customHeight="1" ht="16" r="182" s="53"/>
+    <row customHeight="1" ht="16" r="183" s="53"/>
+    <row customHeight="1" ht="16" r="184" s="53"/>
+    <row customHeight="1" ht="16" r="185" s="53"/>
+    <row customHeight="1" ht="16" r="186" s="53"/>
+    <row customHeight="1" ht="16" r="187" s="53"/>
+    <row customHeight="1" ht="16" r="188" s="53"/>
+    <row customHeight="1" ht="16" r="189" s="53"/>
+    <row customHeight="1" ht="16" r="190" s="53"/>
+    <row customHeight="1" ht="16" r="191" s="53"/>
+    <row customHeight="1" ht="16" r="192" s="53"/>
+    <row customHeight="1" ht="16" r="193" s="53"/>
+    <row customHeight="1" ht="16" r="194" s="53"/>
+    <row customHeight="1" ht="16" r="195" s="53"/>
+    <row customHeight="1" ht="16" r="196" s="53"/>
+    <row customHeight="1" ht="16" r="197" s="53"/>
+    <row customHeight="1" ht="16" r="198" s="53"/>
+    <row customHeight="1" ht="16" r="199" s="53"/>
+    <row customHeight="1" ht="16" r="200" s="53"/>
+    <row customHeight="1" ht="16" r="201" s="53"/>
+    <row customHeight="1" ht="16" r="202" s="53"/>
+    <row customHeight="1" ht="16" r="203" s="53"/>
+    <row customHeight="1" ht="16" r="204" s="53"/>
+    <row customHeight="1" ht="16" r="205" s="53"/>
+    <row customHeight="1" ht="16" r="206" s="53"/>
+    <row customHeight="1" ht="16" r="207" s="53"/>
+    <row customHeight="1" ht="16" r="208" s="53"/>
+    <row customHeight="1" ht="16" r="209" s="53"/>
+    <row customHeight="1" ht="16" r="210" s="53"/>
+    <row customHeight="1" ht="16" r="211" s="53"/>
+    <row customHeight="1" ht="16" r="212" s="53"/>
+    <row customHeight="1" ht="16" r="213" s="53"/>
+    <row customHeight="1" ht="16" r="214" s="53"/>
+    <row customHeight="1" ht="16" r="215" s="53"/>
+    <row customHeight="1" ht="16" r="216" s="53"/>
+    <row customHeight="1" ht="16" r="217" s="53"/>
+    <row customHeight="1" ht="16" r="218" s="53"/>
+    <row customHeight="1" ht="16" r="219" s="53"/>
+    <row customHeight="1" ht="16" r="220" s="53"/>
+    <row customHeight="1" ht="16" r="221" s="53"/>
+    <row customHeight="1" ht="16" r="222" s="53"/>
+    <row customHeight="1" ht="16" r="223" s="53"/>
+    <row customHeight="1" ht="16" r="224" s="53"/>
+    <row customHeight="1" ht="16" r="225" s="53"/>
+    <row customHeight="1" ht="16" r="226" s="53"/>
+    <row customHeight="1" ht="16" r="227" s="53"/>
+    <row customHeight="1" ht="16" r="228" s="53"/>
+    <row customHeight="1" ht="16" r="229" s="53"/>
+    <row customHeight="1" ht="16" r="230" s="53"/>
+    <row customHeight="1" ht="16" r="231" s="53"/>
+    <row customHeight="1" ht="16" r="232" s="53"/>
+    <row customHeight="1" ht="16" r="233" s="53"/>
+    <row customHeight="1" ht="16" r="234" s="53"/>
+    <row customHeight="1" ht="16" r="235" s="53"/>
+    <row customHeight="1" ht="16" r="236" s="53"/>
+    <row customHeight="1" ht="16" r="237" s="53"/>
+    <row customHeight="1" ht="16" r="238" s="53"/>
+    <row customHeight="1" ht="16" r="239" s="53"/>
+    <row customHeight="1" ht="16" r="240" s="53"/>
+    <row customHeight="1" ht="16" r="241" s="53"/>
+    <row customHeight="1" ht="16" r="242" s="53"/>
+    <row customHeight="1" ht="16" r="243" s="53"/>
+    <row customHeight="1" ht="16" r="244" s="53"/>
+    <row customHeight="1" ht="16" r="245" s="53"/>
+    <row customHeight="1" ht="16" r="246" s="53"/>
+    <row customHeight="1" ht="16" r="247" s="53"/>
+    <row customHeight="1" ht="16" r="248" s="53"/>
+    <row customHeight="1" ht="16" r="249" s="53"/>
+    <row customHeight="1" ht="16" r="250" s="53"/>
+    <row customHeight="1" ht="16" r="251" s="53"/>
+    <row customHeight="1" ht="16" r="252" s="53"/>
+    <row customHeight="1" ht="16" r="253" s="53"/>
+    <row customHeight="1" ht="16" r="254" s="53"/>
+    <row customHeight="1" ht="16" r="255" s="53"/>
+    <row customHeight="1" ht="16" r="256" s="53"/>
+    <row customHeight="1" ht="16" r="257" s="53"/>
+    <row customHeight="1" ht="16" r="258" s="53"/>
+    <row customHeight="1" ht="16" r="259" s="53"/>
+    <row customHeight="1" ht="16" r="260" s="53"/>
+    <row customHeight="1" ht="16" r="261" s="53"/>
+    <row customHeight="1" ht="16" r="262" s="53"/>
   </sheetData>
   <autoFilter ref="A2:F61"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -4994,17 +4994,17 @@
   <dimension ref="A1:T207"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -5027,7 +5027,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>区域</t>
@@ -5113,7 +5113,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5156,7 +5156,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5201,7 +5201,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5238,7 +5238,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -5283,7 +5283,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5322,7 +5322,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5359,7 +5359,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5388,7 +5388,7 @@
       <c r="S9" s="14" t="n"/>
       <c r="T9" s="2" t="n"/>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -5427,7 +5427,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5464,7 +5464,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5501,7 +5501,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5540,7 +5540,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5577,7 +5577,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -5604,7 +5604,7 @@
       <c r="N15" s="10" t="n"/>
       <c r="O15" s="10" t="n"/>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5632,7 +5632,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5660,7 +5660,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -5688,7 +5688,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5718,7 +5718,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5748,7 +5748,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5784,7 +5784,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5812,7 +5812,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -5842,7 +5842,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5880,7 +5880,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5910,7 +5910,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -5942,7 +5942,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -5976,7 +5976,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -6008,7 +6008,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6036,7 +6036,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6072,7 +6072,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6099,7 +6099,7 @@
       <c r="N31" s="10" t="n"/>
       <c r="O31" s="10" t="n"/>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6131,7 +6131,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6163,7 +6163,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -6188,7 +6188,7 @@
       <c r="N34" s="10" t="n"/>
       <c r="O34" s="10" t="n"/>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6218,7 +6218,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6248,7 +6248,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6282,7 +6282,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6312,7 +6312,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6340,7 +6340,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6368,7 +6368,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6396,7 +6396,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -6424,7 +6424,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6452,7 +6452,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6480,7 +6480,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6508,7 +6508,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -6536,7 +6536,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6574,7 +6574,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6604,7 +6604,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6640,7 +6640,7 @@
         <v/>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="8" t="inlineStr">
         <is>
           <t>华中区</t>
@@ -6674,7 +6674,7 @@
         <v/>
       </c>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6710,7 +6710,7 @@
         <v/>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -6742,7 +6742,7 @@
         <v/>
       </c>
     </row>
-    <row r="53" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="53" s="53">
       <c r="A53" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -7390,7 +7390,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -7403,17 +7403,17 @@
   <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <cols>
-    <col width="6.33203125" customWidth="1" style="53" min="1" max="1"/>
-    <col width="11.83203125" customWidth="1" style="53" min="2" max="2"/>
-    <col width="3.1640625" customWidth="1" style="17" min="3" max="5"/>
-    <col width="3.1640625" customWidth="1" style="53" min="6" max="11"/>
-    <col width="3.83203125" customWidth="1" style="53" min="12" max="14"/>
-    <col width="3.6640625" customWidth="1" style="53" min="15" max="15"/>
-    <col width="7.6640625" customWidth="1" style="53" min="19" max="19"/>
-    <col width="2.83203125" customWidth="1" style="53" min="20" max="20"/>
+    <col customWidth="1" max="1" min="1" style="53" width="6.33203125"/>
+    <col customWidth="1" max="2" min="2" style="53" width="11.83203125"/>
+    <col customWidth="1" max="5" min="3" style="17" width="3.1640625"/>
+    <col customWidth="1" max="11" min="6" style="53" width="3.1640625"/>
+    <col customWidth="1" max="14" min="12" style="53" width="3.83203125"/>
+    <col customWidth="1" max="15" min="15" style="53" width="3.6640625"/>
+    <col customWidth="1" max="19" min="19" style="53" width="7.6640625"/>
+    <col customWidth="1" max="20" min="20" style="53" width="2.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22.5" customHeight="1" s="53">
+    <row customHeight="1" ht="22.5" r="1" s="53">
       <c r="A1" s="80" t="inlineStr">
         <is>
           <t>2025未填写月报次数</t>
@@ -7436,7 +7436,7 @@
       <c r="S1" s="1" t="n"/>
       <c r="T1" s="2" t="n"/>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="18" t="inlineStr">
         <is>
           <t>区域</t>
@@ -7522,7 +7522,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7568,7 +7568,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7605,7 +7605,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7651,7 +7651,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="8" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -7697,7 +7697,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7745,7 +7745,7 @@
         <v/>
       </c>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7782,7 +7782,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7819,7 +7819,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="8" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -7867,7 +7867,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7913,7 +7913,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7950,7 +7950,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -7987,7 +7987,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8033,7 +8033,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="8" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -8061,7 +8061,7 @@
         <v/>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8089,7 +8089,7 @@
         <v/>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8117,7 +8117,7 @@
         <v/>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="8" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -8145,7 +8145,7 @@
         <v/>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8173,7 +8173,7 @@
         <v/>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8201,7 +8201,7 @@
         <v/>
       </c>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8229,7 +8229,7 @@
         <v/>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8257,7 +8257,7 @@
         <v/>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="8" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -8285,7 +8285,7 @@
         <v/>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8313,7 +8313,7 @@
         <v/>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8341,7 +8341,7 @@
         <v/>
       </c>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="8" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -8369,7 +8369,7 @@
         <v/>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8397,7 +8397,7 @@
         <v/>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="8" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -8427,7 +8427,7 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8455,7 +8455,7 @@
         <v/>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8483,7 +8483,7 @@
         <v/>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8511,7 +8511,7 @@
         <v/>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8539,7 +8539,7 @@
         <v/>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8567,7 +8567,7 @@
         <v/>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="8" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -8595,7 +8595,7 @@
         <v/>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8625,7 +8625,7 @@
         <v/>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8653,7 +8653,7 @@
         <v/>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8681,7 +8681,7 @@
         <v/>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8709,7 +8709,7 @@
         <v/>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8737,7 +8737,7 @@
         <v/>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8767,7 +8767,7 @@
         <v/>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8799,7 +8799,7 @@
         <v/>
       </c>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="8" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -8827,7 +8827,7 @@
         <v/>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8855,7 +8855,7 @@
         <v/>
       </c>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8883,7 +8883,7 @@
         <v/>
       </c>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8911,7 +8911,7 @@
         <v/>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="8" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -8939,7 +8939,7 @@
         <v/>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -8971,7 +8971,7 @@
         <v/>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9003,7 +9003,7 @@
         <v/>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="8" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -9679,7 +9679,7 @@
   <mergeCells count="1">
     <mergeCell ref="A1:O1"/>
   </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -9690,16 +9690,16 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:M57"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10" defaultRowHeight="16.5" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10" defaultRowHeight="16.5"/>
   <cols>
-    <col width="13.1640625" customWidth="1" style="53" min="2" max="2"/>
-    <col width="30.6640625" customWidth="1" style="29" min="4" max="4"/>
-    <col width="26.33203125" customWidth="1" style="30" min="5" max="5"/>
-    <col hidden="1" width="10" customWidth="1" style="53" min="7" max="8"/>
-    <col width="20" customWidth="1" style="53" min="10" max="10"/>
+    <col customWidth="1" max="2" min="2" style="53" width="13.1640625"/>
+    <col customWidth="1" max="4" min="4" style="29" width="30.6640625"/>
+    <col customWidth="1" max="5" min="5" style="30" width="26.33203125"/>
+    <col customWidth="1" hidden="1" max="8" min="7" style="53" width="10"/>
+    <col customWidth="1" max="10" min="10" style="53" width="20"/>
   </cols>
   <sheetData>
-    <row r="1" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="1" s="53">
       <c r="A1" s="0" t="inlineStr">
         <is>
           <t>更新日期</t>
@@ -9709,7 +9709,7 @@
         <v>46121</v>
       </c>
     </row>
-    <row r="2" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="2" s="53">
       <c r="A2" s="27" t="inlineStr">
         <is>
           <t>区域</t>
@@ -9754,7 +9754,7 @@
         <v/>
       </c>
     </row>
-    <row r="3" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="3" s="53">
       <c r="A3" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9800,7 +9800,7 @@
         <v/>
       </c>
     </row>
-    <row r="4" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="4" s="53">
       <c r="A4" s="31" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9845,7 +9845,7 @@
         <v/>
       </c>
     </row>
-    <row r="5" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="5" s="53">
       <c r="A5" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9894,7 +9894,7 @@
         <v/>
       </c>
     </row>
-    <row r="6" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="6" s="53">
       <c r="A6" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9943,7 +9943,7 @@
         <v/>
       </c>
     </row>
-    <row r="7" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="7" s="53">
       <c r="A7" s="37" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -9985,7 +9985,7 @@
       <c r="L7" s="34" t="n"/>
       <c r="M7" s="35" t="n"/>
     </row>
-    <row r="8" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="8" s="53">
       <c r="A8" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10020,7 +10020,7 @@
         <v/>
       </c>
     </row>
-    <row r="9" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="9" s="53">
       <c r="A9" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10060,7 +10060,7 @@
         <v/>
       </c>
     </row>
-    <row r="10" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="10" s="53">
       <c r="A10" s="31" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -10096,7 +10096,7 @@
         <v/>
       </c>
     </row>
-    <row r="11" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="11" s="53">
       <c r="A11" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10132,7 +10132,7 @@
         <v/>
       </c>
     </row>
-    <row r="12" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="12" s="53">
       <c r="A12" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10168,7 +10168,7 @@
         <v/>
       </c>
     </row>
-    <row r="13" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="13" s="53">
       <c r="A13" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10209,7 +10209,7 @@
         <v/>
       </c>
     </row>
-    <row r="14" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="14" s="53">
       <c r="A14" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10240,7 +10240,7 @@
         <v/>
       </c>
     </row>
-    <row r="15" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="15" s="53">
       <c r="A15" s="31" t="inlineStr">
         <is>
           <t>华南三区</t>
@@ -10262,7 +10262,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="16" s="53">
       <c r="A16" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10279,7 +10279,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="17" s="53">
       <c r="A17" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10296,7 +10296,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="18" s="53">
       <c r="A18" s="31" t="inlineStr">
         <is>
           <t>华南四区</t>
@@ -10318,7 +10318,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="19" s="53">
       <c r="A19" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10335,7 +10335,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="20" s="53">
       <c r="A20" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10353,7 +10353,7 @@
       </c>
       <c r="D20" s="39" t="n"/>
     </row>
-    <row r="21" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="21" s="53">
       <c r="A21" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10375,7 +10375,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="22" s="53">
       <c r="A22" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10397,7 +10397,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="23" s="53">
       <c r="A23" s="31" t="inlineStr">
         <is>
           <t>华东一区</t>
@@ -10419,7 +10419,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="24" s="53">
       <c r="A24" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10441,7 +10441,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="25" s="53">
       <c r="A25" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10459,7 +10459,7 @@
       </c>
       <c r="D25" s="36" t="n"/>
     </row>
-    <row r="26" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="26" s="53">
       <c r="A26" s="31" t="inlineStr">
         <is>
           <t>华东二区</t>
@@ -10481,7 +10481,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="27" s="53">
       <c r="A27" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10503,7 +10503,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="28" s="53">
       <c r="A28" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10525,7 +10525,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="29" s="53">
       <c r="A29" s="31" t="inlineStr">
         <is>
           <t>华东三区</t>
@@ -10547,7 +10547,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="30" s="53">
       <c r="A30" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10569,7 +10569,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="31" s="53">
       <c r="A31" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10591,7 +10591,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="32" s="53">
       <c r="A32" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10618,7 +10618,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="33" s="53">
       <c r="A33" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10640,7 +10640,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="34" s="53">
       <c r="A34" s="31" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -10662,7 +10662,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="35" s="53">
       <c r="A35" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10684,7 +10684,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="36" s="53">
       <c r="A36" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10706,7 +10706,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="37" s="53">
       <c r="A37" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10728,7 +10728,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="38" s="53">
       <c r="A38" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10750,7 +10750,7 @@
         </is>
       </c>
     </row>
-    <row r="39" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="39" s="53">
       <c r="A39" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10767,7 +10767,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="40" s="53">
       <c r="A40" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10789,7 +10789,7 @@
         </is>
       </c>
     </row>
-    <row r="41" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="41" s="53">
       <c r="A41" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10807,7 +10807,7 @@
       </c>
       <c r="D41" s="46" t="n"/>
     </row>
-    <row r="42" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="42" s="53">
       <c r="A42" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10829,7 +10829,7 @@
         </is>
       </c>
     </row>
-    <row r="43" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="43" s="53">
       <c r="A43" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10847,7 +10847,7 @@
       </c>
       <c r="D43" s="46" t="n"/>
     </row>
-    <row r="44" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="44" s="53">
       <c r="A44" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10865,7 +10865,7 @@
       </c>
       <c r="E44" s="46" t="n"/>
     </row>
-    <row r="45" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="45" s="53">
       <c r="A45" s="31" t="inlineStr">
         <is>
           <t>华北一区</t>
@@ -10887,7 +10887,7 @@
         </is>
       </c>
     </row>
-    <row r="46" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="46" s="53">
       <c r="A46" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10909,7 +10909,7 @@
         </is>
       </c>
     </row>
-    <row r="47" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="47" s="53">
       <c r="A47" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10931,7 +10931,7 @@
         </is>
       </c>
     </row>
-    <row r="48" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="48" s="53">
       <c r="A48" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10953,7 +10953,7 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="49" s="53">
       <c r="A49" s="31" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -10975,7 +10975,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="50" s="53">
       <c r="A50" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -10998,7 +10998,7 @@
       </c>
       <c r="E50" s="49" t="n"/>
     </row>
-    <row r="51" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="51" s="53">
       <c r="A51" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -11020,7 +11020,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="52" s="53">
       <c r="A52" s="31" t="inlineStr">
         <is>
           <t>西南区</t>
@@ -11042,7 +11042,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="16" customHeight="1" s="53">
+    <row customHeight="1" ht="16" r="53" s="53">
       <c r="A53" s="37" t="inlineStr">
         <is>
           <t>华南二区</t>
@@ -11064,7 +11064,7 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="54" s="53">
       <c r="A54" s="55" t="inlineStr">
         <is>
           <t>华南一区</t>
@@ -11086,7 +11086,7 @@
         </is>
       </c>
     </row>
-    <row r="55" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="55" s="53">
       <c r="A55" s="55" t="inlineStr">
         <is>
           <t>华东四区</t>
@@ -11108,7 +11108,7 @@
         </is>
       </c>
     </row>
-    <row r="56" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="56" s="53">
       <c r="A56" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11130,7 +11130,7 @@
         </is>
       </c>
     </row>
-    <row r="57" ht="16.5" customHeight="1" s="53">
+    <row customHeight="1" ht="16.5" r="57" s="53">
       <c r="A57" s="55" t="inlineStr">
         <is>
           <t>华北二区</t>
@@ -11148,7 +11148,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
 
@@ -11159,18 +11159,18 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I38"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" customHeight="1" defaultColWidth="10.83203125" defaultRowHeight="15"/>
   <cols>
-    <col width="6.83203125" customWidth="1" style="23" min="1" max="1"/>
-    <col width="8.83203125" customWidth="1" style="23" min="2" max="2"/>
-    <col width="19.6640625" customWidth="1" style="23" min="3" max="3"/>
-    <col width="13" customWidth="1" style="23" min="4" max="4"/>
-    <col hidden="1" width="30.5" customWidth="1" style="23" min="5" max="6"/>
-    <col width="30.5" customWidth="1" style="23" min="7" max="7"/>
-    <col width="10.83203125" customWidth="1" style="23" min="8" max="26"/>
+    <col customWidth="1" max="1" min="1" style="23" width="6.83203125"/>
+    <col customWidth="1" max="2" min="2" style="23" width="8.83203125"/>
+    <col customWidth="1" max="3" min="3" style="23" width="19.6640625"/>
+    <col customWidth="1" max="4" min="4" style="23" width="13"/>
+    <col customWidth="1" hidden="1" max="6" min="5" style="23" width="30.5"/>
+    <col customWidth="1" max="7" min="7" style="23" width="30.5"/>
+    <col customWidth="1" max="26" min="8" style="23" width="10.83203125"/>
   </cols>
   <sheetData>
-    <row r="1" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="1" s="53">
       <c r="A1" s="21" t="n"/>
       <c r="B1" s="22" t="inlineStr">
         <is>
@@ -11212,7 +11212,7 @@
         <v/>
       </c>
     </row>
-    <row r="2" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="2" s="53">
       <c r="A2" s="24" t="n">
         <v>1</v>
       </c>
@@ -11255,7 +11255,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="3" s="53">
       <c r="A3" s="24" t="n">
         <v>2</v>
       </c>
@@ -11288,7 +11288,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="4" s="53">
       <c r="A4" s="24" t="n">
         <v>3</v>
       </c>
@@ -11326,7 +11326,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="5" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="5" s="53">
       <c r="A5" s="24" t="n">
         <v>4</v>
       </c>
@@ -11369,7 +11369,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="6" s="53">
       <c r="A6" s="24" t="n">
         <v>5</v>
       </c>
@@ -11402,7 +11402,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="7" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="7" s="53">
       <c r="A7" s="24" t="n">
         <v>6</v>
       </c>
@@ -11431,7 +11431,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="8" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="8" s="53">
       <c r="A8" s="24" t="n">
         <v>7</v>
       </c>
@@ -11461,7 +11461,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="9" s="53">
       <c r="A9" s="24" t="n">
         <v>8</v>
       </c>
@@ -11486,7 +11486,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="10" s="53">
       <c r="A10" s="24" t="n">
         <v>1</v>
       </c>
@@ -11511,7 +11511,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="11" s="53">
       <c r="A11" s="24" t="n">
         <v>2</v>
       </c>
@@ -11541,7 +11541,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="12" s="53">
       <c r="A12" s="24" t="n">
         <v>3</v>
       </c>
@@ -11566,7 +11566,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="13" s="53">
       <c r="A13" s="24" t="n">
         <v>4</v>
       </c>
@@ -11596,7 +11596,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="14" s="53">
       <c r="A14" s="24" t="n">
         <v>5</v>
       </c>
@@ -11616,7 +11616,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="15" s="53">
       <c r="A15" s="24" t="n">
         <v>6</v>
       </c>
@@ -11646,7 +11646,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="16" s="53">
       <c r="A16" s="24" t="n">
         <v>1</v>
       </c>
@@ -11671,7 +11671,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="17" s="53">
       <c r="A17" s="24" t="n">
         <v>2</v>
       </c>
@@ -11706,7 +11706,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="18" s="53">
       <c r="A18" s="24" t="n">
         <v>3</v>
       </c>
@@ -11741,7 +11741,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="19" s="53">
       <c r="A19" s="24" t="n">
         <v>4</v>
       </c>
@@ -11766,7 +11766,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="20" s="53">
       <c r="A20" s="24" t="n">
         <v>5</v>
       </c>
@@ -11796,7 +11796,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="21" s="53">
       <c r="A21" s="24" t="n">
         <v>6</v>
       </c>
@@ -11826,7 +11826,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="22" s="53">
       <c r="A22" s="24" t="n">
         <v>7</v>
       </c>
@@ -11856,7 +11856,7 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="23" s="53">
       <c r="A23" s="24" t="n">
         <v>8</v>
       </c>
@@ -11886,7 +11886,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="24" s="53">
       <c r="A24" s="24" t="n">
         <v>1</v>
       </c>
@@ -11916,7 +11916,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="25" s="53">
       <c r="A25" s="24" t="n">
         <v>2</v>
       </c>
@@ -11946,7 +11946,7 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="26" s="53">
       <c r="A26" s="24" t="n">
         <v>3</v>
       </c>
@@ -11971,7 +11971,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="27" s="53">
       <c r="A27" s="24" t="n">
         <v>4</v>
       </c>
@@ -12001,7 +12001,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="28" s="53">
       <c r="A28" s="24" t="n">
         <v>5</v>
       </c>
@@ -12031,7 +12031,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="29" s="53">
       <c r="A29" s="24" t="n">
         <v>6</v>
       </c>
@@ -12061,7 +12061,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="30" s="53">
       <c r="A30" s="24" t="n">
         <v>7</v>
       </c>
@@ -12096,7 +12096,7 @@
         </is>
       </c>
     </row>
-    <row r="31" ht="15.75" customHeight="1" s="53">
+    <row customHeight="1" ht="15.75" r="31" s="53">
       <c r="A31" s="24" t="n">
         <v>8</v>
       </c>
@@ -12126,7 +12126,7 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="32" s="53">
       <c r="A32" s="24" t="n">
         <v>1</v>
       </c>
@@ -12156,7 +12156,7 @@
         </is>
       </c>
     </row>
-    <row r="33" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="33" s="53">
       <c r="A33" s="24" t="n">
         <v>2</v>
       </c>
@@ -12186,7 +12186,7 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="34" s="53">
       <c r="A34" s="24" t="n">
         <v>3</v>
       </c>
@@ -12216,7 +12216,7 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="35" s="53">
       <c r="A35" s="24" t="n">
         <v>4</v>
       </c>
@@ -12246,7 +12246,7 @@
         </is>
       </c>
     </row>
-    <row r="36" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="36" s="53">
       <c r="A36" s="24" t="n">
         <v>1</v>
       </c>
@@ -12276,7 +12276,7 @@
         </is>
       </c>
     </row>
-    <row r="37" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="37" s="53">
       <c r="A37" s="24" t="n">
         <v>2</v>
       </c>
@@ -12311,7 +12311,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="15" customHeight="1" s="53">
+    <row customHeight="1" ht="15" r="38" s="53">
       <c r="A38" s="24" t="n">
         <v>3</v>
       </c>
@@ -12342,6 +12342,6 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
report: update 2026-10-30 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46324</v>
+        <v>46325</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -4249,7 +4249,7 @@
       </c>
       <c r="D48" s="71" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发2次，迟发3次</t>
         </is>
       </c>
       <c r="E48" s="69" t="n"/>
@@ -4444,7 +4444,7 @@
       </c>
       <c r="D55" s="70" t="inlineStr">
         <is>
-          <t>累计未发5次，迟发3次</t>
+          <t>累计未发5次，迟发4次</t>
         </is>
       </c>
       <c r="E55" s="69" t="n"/>
@@ -4775,7 +4775,7 @@
       </c>
       <c r="D67" s="0" t="inlineStr">
         <is>
-          <t>累计未发2次</t>
+          <t>累计未发3次</t>
         </is>
       </c>
       <c r="F67" s="0" t="inlineStr">

</xml_diff>

<commit_message>
report: update 2026-10-31 daily status
</commit_message>
<xml_diff>
--- a/日报及月报发送记录.xlsx
+++ b/日报及月报发送记录.xlsx
@@ -2635,7 +2635,7 @@
         </is>
       </c>
       <c r="B1" s="52" t="n">
-        <v>46325</v>
+        <v>46326</v>
       </c>
     </row>
     <row customHeight="1" ht="16.5" r="2" s="53">
@@ -3971,7 +3971,7 @@
       </c>
       <c r="D38" s="68" t="inlineStr">
         <is>
-          <t>累计未发2次，迟发2次</t>
+          <t>累计未发3次，迟发2次</t>
         </is>
       </c>
       <c r="E38" s="69" t="n"/>

</xml_diff>